<commit_message>
h5 reader to technologies.xlsx
</commit_message>
<xml_diff>
--- a/case_studies/current_layout/technologies.xlsx
+++ b/case_studies/current_layout/technologies.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Github\AdOpT-NET0_my\case_studies\backbone_2026\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Github\AdOpT-NET0_my\case_studies\current_layout\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16B7F995-16AD-4DF2-925D-4F55DD5167F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C82AA6A8-DE5A-40F5-A7C3-C8D0A9DA358B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="existing" sheetId="3" r:id="rId1"/>
@@ -1246,7 +1246,7 @@
         <v>0</v>
       </c>
       <c r="T2">
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="U2">
         <v>0</v>
@@ -1261,6 +1261,9 @@
         <v>0</v>
       </c>
       <c r="Y2">
+        <v>0</v>
+      </c>
+      <c r="Z2">
         <v>0</v>
       </c>
     </row>
@@ -1340,6 +1343,9 @@
       <c r="Y3">
         <v>0</v>
       </c>
+      <c r="Z3">
+        <v>45</v>
+      </c>
     </row>
     <row r="4" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
@@ -1367,13 +1373,13 @@
         <v>0</v>
       </c>
       <c r="I4">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="J4">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="K4">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="L4">
         <v>0</v>
@@ -1400,7 +1406,7 @@
         <v>0</v>
       </c>
       <c r="T4">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="U4">
         <v>0</v>
@@ -1416,6 +1422,9 @@
       </c>
       <c r="Y4">
         <v>0</v>
+      </c>
+      <c r="Z4">
+        <v>39</v>
       </c>
     </row>
     <row r="5" spans="1:26" x14ac:dyDescent="0.3">
@@ -1450,7 +1459,7 @@
         <v>79</v>
       </c>
       <c r="K5">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="L5">
         <v>0</v>
@@ -1493,6 +1502,9 @@
       </c>
       <c r="Y5">
         <v>0</v>
+      </c>
+      <c r="Z5">
+        <v>212</v>
       </c>
     </row>
     <row r="6" spans="1:26" x14ac:dyDescent="0.3">
@@ -1521,13 +1533,13 @@
         <v>0</v>
       </c>
       <c r="I6">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="J6">
-        <v>62</v>
+        <v>47</v>
       </c>
       <c r="K6">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="L6">
         <v>0</v>
@@ -1554,7 +1566,7 @@
         <v>0</v>
       </c>
       <c r="T6">
-        <v>12</v>
+        <v>32</v>
       </c>
       <c r="U6">
         <v>0</v>
@@ -1569,6 +1581,9 @@
         <v>0</v>
       </c>
       <c r="Y6">
+        <v>0</v>
+      </c>
+      <c r="Z6">
         <v>0</v>
       </c>
     </row>
@@ -1648,6 +1663,9 @@
       <c r="Y7">
         <v>0</v>
       </c>
+      <c r="Z7">
+        <v>0</v>
+      </c>
     </row>
     <row r="8" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
@@ -1708,7 +1726,7 @@
         <v>0</v>
       </c>
       <c r="T8">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="U8">
         <v>0</v>
@@ -1723,6 +1741,9 @@
         <v>0</v>
       </c>
       <c r="Y8">
+        <v>0</v>
+      </c>
+      <c r="Z8">
         <v>0</v>
       </c>
     </row>

</xml_diff>